<commit_message>
Update figure names, improve tables formatting
</commit_message>
<xml_diff>
--- a/Table S1 - FoldSeek results for the designed protein.xlsx
+++ b/Table S1 - FoldSeek results for the designed protein.xlsx
@@ -66,7 +66,7 @@
     <t xml:space="preserve">Target Pos. (Len)</t>
   </si>
   <si>
-    <t xml:space="preserve">5a8w</t>
+    <t xml:space="preserve">5A8W</t>
   </si>
   <si>
     <t xml:space="preserve"> Methanothermobacter wolfeii </t>
@@ -78,7 +78,7 @@
     <t xml:space="preserve">299-524 (549)</t>
   </si>
   <si>
-    <t xml:space="preserve">5n1q</t>
+    <t xml:space="preserve">5N1Q</t>
   </si>
   <si>
     <t xml:space="preserve"> Methanothermococcus thermolithotrophicus DSM 2095 </t>
@@ -90,7 +90,7 @@
     <t xml:space="preserve">298-496 (549)</t>
   </si>
   <si>
-    <t xml:space="preserve">1e6y</t>
+    <t xml:space="preserve">1E6Y</t>
   </si>
   <si>
     <t xml:space="preserve"> Methanosarcina barkeri </t>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">311-543 (568)</t>
   </si>
   <si>
-    <t xml:space="preserve">3m1v</t>
+    <t xml:space="preserve">3M1V</t>
   </si>
   <si>
     <t xml:space="preserve"> Methanothermobacter marburgensis str. Marburg </t>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">298-496 (548)</t>
   </si>
   <si>
-    <t xml:space="preserve">7qpi</t>
+    <t xml:space="preserve">7QPI</t>
   </si>
   <si>
     <t xml:space="preserve"> Petromyzon marinus </t>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">13-208 (238)</t>
   </si>
   <si>
-    <t xml:space="preserve">5dks</t>
+    <t xml:space="preserve">5DKS</t>
   </si>
   <si>
     <t xml:space="preserve"> Homo sapiens </t>
@@ -132,13 +132,13 @@
     <t xml:space="preserve">12-201 (225)</t>
   </si>
   <si>
-    <t xml:space="preserve">5u2b</t>
+    <t xml:space="preserve">5U2B</t>
   </si>
   <si>
     <t xml:space="preserve">18-218 (242)</t>
   </si>
   <si>
-    <t xml:space="preserve">7zu1</t>
+    <t xml:space="preserve">7ZU1</t>
   </si>
   <si>
     <t xml:space="preserve">4-113 (120)</t>
@@ -147,7 +147,7 @@
     <t xml:space="preserve">4-240 (245)</t>
   </si>
   <si>
-    <t xml:space="preserve">4tq3</t>
+    <t xml:space="preserve">4TQ3</t>
   </si>
   <si>
     <t xml:space="preserve"> Archaeoglobus fulgidus DSM 4304 </t>
@@ -156,7 +156,7 @@
     <t xml:space="preserve">13-268 (283)</t>
   </si>
   <si>
-    <t xml:space="preserve">6lcn</t>
+    <t xml:space="preserve">6LCN</t>
   </si>
   <si>
     <t xml:space="preserve"> Planctopirus limnophila DSM 3776 </t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">30-216 (294)</t>
   </si>
   <si>
-    <t xml:space="preserve">3ce9</t>
+    <t xml:space="preserve">3CE9</t>
   </si>
   <si>
     <t xml:space="preserve"> Clostridium acetobutylicum ATCC 824 </t>
@@ -180,7 +180,7 @@
     <t xml:space="preserve">174-336 (348)</t>
   </si>
   <si>
-    <t xml:space="preserve">3ejz</t>
+    <t xml:space="preserve">3EJZ</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia coli </t>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">230-422 (444)</t>
   </si>
   <si>
-    <t xml:space="preserve">8gf6</t>
+    <t xml:space="preserve">8GF6</t>
   </si>
   <si>
     <t xml:space="preserve"> Methanosarcina acetivorans C2A </t>
@@ -204,19 +204,19 @@
     <t xml:space="preserve">216-439 (461)</t>
   </si>
   <si>
-    <t xml:space="preserve">5jy3</t>
+    <t xml:space="preserve">5JY3</t>
   </si>
   <si>
     <t xml:space="preserve">13-209 (231)</t>
   </si>
   <si>
-    <t xml:space="preserve">3tx7</t>
+    <t xml:space="preserve">3TX7</t>
   </si>
   <si>
     <t xml:space="preserve">10-191 (218)</t>
   </si>
   <si>
-    <t xml:space="preserve">4n6b</t>
+    <t xml:space="preserve">4N6B</t>
   </si>
   <si>
     <t xml:space="preserve"> Glycine max </t>
@@ -228,13 +228,13 @@
     <t xml:space="preserve">51-161 (232)</t>
   </si>
   <si>
-    <t xml:space="preserve">4tq5</t>
+    <t xml:space="preserve">4TQ5</t>
   </si>
   <si>
     <t xml:space="preserve">13-260 (275)</t>
   </si>
   <si>
-    <t xml:space="preserve">3pde</t>
+    <t xml:space="preserve">3PDE</t>
   </si>
   <si>
     <t xml:space="preserve"> Levilactobacillus brevis ATCC 367 </t>
@@ -246,13 +246,13 @@
     <t xml:space="preserve">47-283 (287)</t>
   </si>
   <si>
-    <t xml:space="preserve">7axe</t>
+    <t xml:space="preserve">7AXE</t>
   </si>
   <si>
     <t xml:space="preserve">1-222 (276)</t>
   </si>
   <si>
-    <t xml:space="preserve">7buu</t>
+    <t xml:space="preserve">7BUU</t>
   </si>
   <si>
     <t xml:space="preserve"> Eucommia ulmoides </t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">47-333 (338)</t>
   </si>
   <si>
-    <t xml:space="preserve">6yze</t>
+    <t xml:space="preserve">6YZE</t>
   </si>
   <si>
     <t xml:space="preserve"> Legionella pneumophila </t>
@@ -273,7 +273,7 @@
     <t xml:space="preserve">109-307 (328)</t>
   </si>
   <si>
-    <t xml:space="preserve">6lsc</t>
+    <t xml:space="preserve">6LSC</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia coli K-12 </t>
@@ -282,7 +282,7 @@
     <t xml:space="preserve">212-399 (423)</t>
   </si>
   <si>
-    <t xml:space="preserve">2oqb</t>
+    <t xml:space="preserve">2OQB</t>
   </si>
   <si>
     <t xml:space="preserve"> Rattus norvegicus </t>
@@ -291,7 +291,7 @@
     <t xml:space="preserve">11-91 (106)</t>
   </si>
   <si>
-    <t xml:space="preserve">7qwv</t>
+    <t xml:space="preserve">7QWV</t>
   </si>
   <si>
     <t xml:space="preserve"> Mus musculus </t>
@@ -300,7 +300,7 @@
     <t xml:space="preserve">9-91 (117)</t>
   </si>
   <si>
-    <t xml:space="preserve">1sst</t>
+    <t xml:space="preserve">1SST</t>
   </si>
   <si>
     <t xml:space="preserve"> Haemophilus influenzae </t>
@@ -312,7 +312,7 @@
     <t xml:space="preserve">53-167 (233)</t>
   </si>
   <si>
-    <t xml:space="preserve">4ny9</t>
+    <t xml:space="preserve">4NY9</t>
   </si>
   <si>
     <t xml:space="preserve">16-120 (120)</t>
@@ -321,7 +321,7 @@
     <t xml:space="preserve">9-209 (260)</t>
   </si>
   <si>
-    <t xml:space="preserve">8szv</t>
+    <t xml:space="preserve">8SZV</t>
   </si>
   <si>
     <t xml:space="preserve">17-111 (120)</t>
@@ -330,7 +330,7 @@
     <t xml:space="preserve">9-246 (274)</t>
   </si>
   <si>
-    <t xml:space="preserve">1nrl</t>
+    <t xml:space="preserve">1NRL</t>
   </si>
   <si>
     <t xml:space="preserve">17-120 (120)</t>
@@ -339,19 +339,19 @@
     <t xml:space="preserve">9-220 (275)</t>
   </si>
   <si>
-    <t xml:space="preserve">7axi</t>
+    <t xml:space="preserve">7AXI</t>
   </si>
   <si>
     <t xml:space="preserve">9-214 (272)</t>
   </si>
   <si>
-    <t xml:space="preserve">6nx1</t>
+    <t xml:space="preserve">6NX1</t>
   </si>
   <si>
     <t xml:space="preserve">10-221 (288)</t>
   </si>
   <si>
-    <t xml:space="preserve">4s0t</t>
+    <t xml:space="preserve">4S0T</t>
   </si>
   <si>
     <t xml:space="preserve">9-232 (283)</t>
@@ -366,7 +366,7 @@
     <t xml:space="preserve">8-257 (279)</t>
   </si>
   <si>
-    <t xml:space="preserve">5fb3</t>
+    <t xml:space="preserve">5FB3</t>
   </si>
   <si>
     <t xml:space="preserve"> Pyrobaculum calidifontis JCM 11548 </t>
@@ -375,7 +375,7 @@
     <t xml:space="preserve">158-315 (329)</t>
   </si>
   <si>
-    <t xml:space="preserve">4kt5</t>
+    <t xml:space="preserve">4KT5</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia coli O157:H7 </t>
@@ -384,13 +384,13 @@
     <t xml:space="preserve">8-106 (114)</t>
   </si>
   <si>
-    <t xml:space="preserve">2ovs</t>
+    <t xml:space="preserve">2OVS</t>
   </si>
   <si>
     <t xml:space="preserve">15-113 (118)</t>
   </si>
   <si>
-    <t xml:space="preserve">4wak</t>
+    <t xml:space="preserve">4WAK</t>
   </si>
   <si>
     <t xml:space="preserve"> Haemophilus influenzae Rd KW20 </t>
@@ -402,7 +402,7 @@
     <t xml:space="preserve">32-172 (173)</t>
   </si>
   <si>
-    <t xml:space="preserve">7udo</t>
+    <t xml:space="preserve">7UDO</t>
   </si>
   <si>
     <t xml:space="preserve"> synthetic construct </t>
@@ -414,13 +414,13 @@
     <t xml:space="preserve">4-150 (172)</t>
   </si>
   <si>
-    <t xml:space="preserve">4fp4</t>
+    <t xml:space="preserve">4FP4</t>
   </si>
   <si>
     <t xml:space="preserve">40-230 (234)</t>
   </si>
   <si>
-    <t xml:space="preserve">5k9r</t>
+    <t xml:space="preserve">5K9R</t>
   </si>
   <si>
     <t xml:space="preserve">20-120 (120)</t>
@@ -429,13 +429,13 @@
     <t xml:space="preserve">16-299 (312)</t>
   </si>
   <si>
-    <t xml:space="preserve">5edi</t>
+    <t xml:space="preserve">5EDI</t>
   </si>
   <si>
     <t xml:space="preserve">22-303 (317)</t>
   </si>
   <si>
-    <t xml:space="preserve">4v3i</t>
+    <t xml:space="preserve">4V3I</t>
   </si>
   <si>
     <t xml:space="preserve"> Vibrio cholerae </t>
@@ -447,7 +447,7 @@
     <t xml:space="preserve">1-122 (153)</t>
   </si>
   <si>
-    <t xml:space="preserve">4u9l</t>
+    <t xml:space="preserve">4U9L</t>
   </si>
   <si>
     <t xml:space="preserve"> Thermus thermophilus HB8 </t>
@@ -465,7 +465,7 @@
     <t xml:space="preserve">22-303 (320)</t>
   </si>
   <si>
-    <t xml:space="preserve">3mv2</t>
+    <t xml:space="preserve">3MV2</t>
   </si>
   <si>
     <t xml:space="preserve"> Saccharomyces cerevisiae </t>
@@ -477,7 +477,7 @@
     <t xml:space="preserve">1-241 (293)</t>
   </si>
   <si>
-    <t xml:space="preserve">2kkm</t>
+    <t xml:space="preserve">2KKM</t>
   </si>
   <si>
     <t xml:space="preserve">35-111 (120)</t>
@@ -486,7 +486,7 @@
     <t xml:space="preserve">16-135 (141)</t>
   </si>
   <si>
-    <t xml:space="preserve">7axh</t>
+    <t xml:space="preserve">7AXH</t>
   </si>
   <si>
     <t xml:space="preserve">18-120 (120)</t>
@@ -495,7 +495,7 @@
     <t xml:space="preserve">10-214 (272)</t>
   </si>
   <si>
-    <t xml:space="preserve">2vwa</t>
+    <t xml:space="preserve">2VWA</t>
   </si>
   <si>
     <t xml:space="preserve"> Plasmodium falciparum 3D7 </t>
@@ -507,7 +507,7 @@
     <t xml:space="preserve">16-93 (99)</t>
   </si>
   <si>
-    <t xml:space="preserve">7bqr</t>
+    <t xml:space="preserve">7BQR</t>
   </si>
   <si>
     <t xml:space="preserve">1-94 (120)</t>
@@ -516,7 +516,7 @@
     <t xml:space="preserve">14-110 (137)</t>
   </si>
   <si>
-    <t xml:space="preserve">4nk1</t>
+    <t xml:space="preserve">4NK1</t>
   </si>
   <si>
     <t xml:space="preserve"> Methylacidiphilum infernorum V4 </t>
@@ -525,13 +525,13 @@
     <t xml:space="preserve">12-136 (160)</t>
   </si>
   <si>
-    <t xml:space="preserve">6qf5</t>
+    <t xml:space="preserve">6QF5</t>
   </si>
   <si>
     <t xml:space="preserve">4-207 (220)</t>
   </si>
   <si>
-    <t xml:space="preserve">3c37</t>
+    <t xml:space="preserve">3C37</t>
   </si>
   <si>
     <t xml:space="preserve"> Geobacter sulfurreducens PCA </t>
@@ -543,7 +543,7 @@
     <t xml:space="preserve">49-201 (222)</t>
   </si>
   <si>
-    <t xml:space="preserve">5dl2</t>
+    <t xml:space="preserve">5DL2</t>
   </si>
   <si>
     <t xml:space="preserve"> Streptococcus pyogenes MGAS10870 </t>
@@ -555,19 +555,19 @@
     <t xml:space="preserve">26-216 (222)</t>
   </si>
   <si>
-    <t xml:space="preserve">5x0r</t>
+    <t xml:space="preserve">5X0R</t>
   </si>
   <si>
     <t xml:space="preserve">11-204 (257)</t>
   </si>
   <si>
-    <t xml:space="preserve">5a86</t>
+    <t xml:space="preserve">5A86</t>
   </si>
   <si>
     <t xml:space="preserve">8-215 (271)</t>
   </si>
   <si>
-    <t xml:space="preserve">4mu6</t>
+    <t xml:space="preserve">4MU6</t>
   </si>
   <si>
     <t xml:space="preserve"> Legionella pneumophila subsp. pneumophila str. Philadelphia 1 </t>
@@ -579,7 +579,7 @@
     <t xml:space="preserve">8-274 (274)</t>
   </si>
   <si>
-    <t xml:space="preserve">7axa</t>
+    <t xml:space="preserve">7AXA</t>
   </si>
   <si>
     <t xml:space="preserve">27-120 (120)</t>
@@ -588,19 +588,19 @@
     <t xml:space="preserve">97-243 (272)</t>
   </si>
   <si>
-    <t xml:space="preserve">6dup</t>
+    <t xml:space="preserve">6DUP</t>
   </si>
   <si>
     <t xml:space="preserve">9-208 (280)</t>
   </si>
   <si>
-    <t xml:space="preserve">6bns</t>
+    <t xml:space="preserve">6BNS</t>
   </si>
   <si>
     <t xml:space="preserve">8-212 (283)</t>
   </si>
   <si>
-    <t xml:space="preserve">2zlv</t>
+    <t xml:space="preserve">2ZLV</t>
   </si>
   <si>
     <t xml:space="preserve"> Equus caballus </t>
@@ -612,7 +612,7 @@
     <t xml:space="preserve">2-131 (132)</t>
   </si>
   <si>
-    <t xml:space="preserve">2qls</t>
+    <t xml:space="preserve">2QLS</t>
   </si>
   <si>
     <t xml:space="preserve"> Canis lupus familiaris </t>
@@ -624,7 +624,7 @@
     <t xml:space="preserve">4-145 (146)</t>
   </si>
   <si>
-    <t xml:space="preserve">1yhu</t>
+    <t xml:space="preserve">1YHU</t>
   </si>
   <si>
     <t xml:space="preserve"> Riftia pachyptila </t>
@@ -636,13 +636,13 @@
     <t xml:space="preserve">12-144 (144)</t>
   </si>
   <si>
-    <t xml:space="preserve">3mjp</t>
+    <t xml:space="preserve">3MJP</t>
   </si>
   <si>
     <t xml:space="preserve"> Coturnix japonica </t>
   </si>
   <si>
-    <t xml:space="preserve">1pqj</t>
+    <t xml:space="preserve">1PQJ</t>
   </si>
   <si>
     <t xml:space="preserve"> Tequatrovirus T4 </t>
@@ -654,7 +654,7 @@
     <t xml:space="preserve">25-154 (164)</t>
   </si>
   <si>
-    <t xml:space="preserve">5b6b</t>
+    <t xml:space="preserve">5B6B</t>
   </si>
   <si>
     <t xml:space="preserve">2-104 (120)</t>
@@ -663,7 +663,7 @@
     <t xml:space="preserve">2-172 (173)</t>
   </si>
   <si>
-    <t xml:space="preserve">4kyz</t>
+    <t xml:space="preserve">4KYZ</t>
   </si>
   <si>
     <t xml:space="preserve">1-110 (120)</t>
@@ -672,7 +672,7 @@
     <t xml:space="preserve">1-161 (167)</t>
   </si>
   <si>
-    <t xml:space="preserve">1b8d</t>
+    <t xml:space="preserve">1B8D</t>
   </si>
   <si>
     <t xml:space="preserve"> Griffithsia monilis </t>
@@ -684,7 +684,7 @@
     <t xml:space="preserve">41-176 (176)</t>
   </si>
   <si>
-    <t xml:space="preserve">2vjh</t>
+    <t xml:space="preserve">2VJH</t>
   </si>
   <si>
     <t xml:space="preserve"> Gloeobacter violaceus </t>
@@ -696,7 +696,7 @@
     <t xml:space="preserve">4-175 (177)</t>
   </si>
   <si>
-    <t xml:space="preserve">5b5v</t>
+    <t xml:space="preserve">5B5V</t>
   </si>
   <si>
     <t xml:space="preserve">26-117 (120)</t>
@@ -705,7 +705,7 @@
     <t xml:space="preserve">13-184 (187)</t>
   </si>
   <si>
-    <t xml:space="preserve">7qoe</t>
+    <t xml:space="preserve">7QOE</t>
   </si>
   <si>
     <t xml:space="preserve"> Leptospira levettii </t>
@@ -717,13 +717,13 @@
     <t xml:space="preserve">16-157 (187)</t>
   </si>
   <si>
-    <t xml:space="preserve">7cfo</t>
+    <t xml:space="preserve">7CFO</t>
   </si>
   <si>
     <t xml:space="preserve">17-166 (193)</t>
   </si>
   <si>
-    <t xml:space="preserve">8e4g</t>
+    <t xml:space="preserve">8E4G</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia phage T7 </t>
@@ -741,13 +741,13 @@
     <t xml:space="preserve">45-202 (223)</t>
   </si>
   <si>
-    <t xml:space="preserve">3r8d</t>
+    <t xml:space="preserve">3R8D</t>
   </si>
   <si>
     <t xml:space="preserve">9-209 (264)</t>
   </si>
   <si>
-    <t xml:space="preserve">7ubl</t>
+    <t xml:space="preserve">7UBL</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia phage Lambda </t>
@@ -759,7 +759,7 @@
     <t xml:space="preserve">1-125 (141)</t>
   </si>
   <si>
-    <t xml:space="preserve">1ebt</t>
+    <t xml:space="preserve">1EBT</t>
   </si>
   <si>
     <t xml:space="preserve"> Phacoides pectinatus </t>
@@ -771,13 +771,13 @@
     <t xml:space="preserve">8-134 (142)</t>
   </si>
   <si>
-    <t xml:space="preserve">5brm</t>
+    <t xml:space="preserve">5BRM</t>
   </si>
   <si>
     <t xml:space="preserve">35-150 (158)</t>
   </si>
   <si>
-    <t xml:space="preserve">1paq</t>
+    <t xml:space="preserve">1PAQ</t>
   </si>
   <si>
     <t xml:space="preserve">16-115 (120)</t>
@@ -786,7 +786,7 @@
     <t xml:space="preserve">63-150 (161)</t>
   </si>
   <si>
-    <t xml:space="preserve">5twf</t>
+    <t xml:space="preserve">5TWF</t>
   </si>
   <si>
     <t xml:space="preserve">26-116 (120)</t>
@@ -804,7 +804,7 @@
     <t xml:space="preserve">3-182 (182)</t>
   </si>
   <si>
-    <t xml:space="preserve">4v8m</t>
+    <t xml:space="preserve">4V8M</t>
   </si>
   <si>
     <t xml:space="preserve"> Trypanosoma brucei brucei TREU927 </t>
@@ -816,13 +816,13 @@
     <t xml:space="preserve">15-173 (205)</t>
   </si>
   <si>
-    <t xml:space="preserve">8acy</t>
+    <t xml:space="preserve">8ACY</t>
   </si>
   <si>
     <t xml:space="preserve">1-202 (204)</t>
   </si>
   <si>
-    <t xml:space="preserve">7y1c</t>
+    <t xml:space="preserve">7Y1C</t>
   </si>
   <si>
     <t xml:space="preserve"> Klebsiella phage Kp9 </t>
@@ -834,7 +834,7 @@
     <t xml:space="preserve">42-171 (192)</t>
   </si>
   <si>
-    <t xml:space="preserve">5z5l</t>
+    <t xml:space="preserve">5Z5L</t>
   </si>
   <si>
     <t xml:space="preserve"> Canavalia ensiformis </t>
@@ -846,7 +846,7 @@
     <t xml:space="preserve">3-232 (233)</t>
   </si>
   <si>
-    <t xml:space="preserve">8szo</t>
+    <t xml:space="preserve">8SZO</t>
   </si>
   <si>
     <t xml:space="preserve"> Canavalia villosa </t>
@@ -855,7 +855,7 @@
     <t xml:space="preserve">17-233 (233)</t>
   </si>
   <si>
-    <t xml:space="preserve">4z8b</t>
+    <t xml:space="preserve">4Z8B</t>
   </si>
   <si>
     <t xml:space="preserve"> Macropsychanthus grandiflorus </t>
@@ -867,7 +867,7 @@
     <t xml:space="preserve">21-230 (231)</t>
   </si>
   <si>
-    <t xml:space="preserve">4pcr</t>
+    <t xml:space="preserve">4PCR</t>
   </si>
   <si>
     <t xml:space="preserve"> Canavalia brasiliensis </t>
@@ -876,7 +876,7 @@
     <t xml:space="preserve">22-231 (232)</t>
   </si>
   <si>
-    <t xml:space="preserve">4hbo</t>
+    <t xml:space="preserve">4HBO</t>
   </si>
   <si>
     <t xml:space="preserve"> Rubella virus strain M33 </t>
@@ -885,13 +885,13 @@
     <t xml:space="preserve">1-80 (81)</t>
   </si>
   <si>
-    <t xml:space="preserve">4dr7</t>
+    <t xml:space="preserve">4DR7</t>
   </si>
   <si>
     <t xml:space="preserve">1-86 (88)</t>
   </si>
   <si>
-    <t xml:space="preserve">7m0q</t>
+    <t xml:space="preserve">7M0Q</t>
   </si>
   <si>
     <t xml:space="preserve">3-109 (120)</t>
@@ -900,13 +900,13 @@
     <t xml:space="preserve">5-97 (97)</t>
   </si>
   <si>
-    <t xml:space="preserve">4har</t>
+    <t xml:space="preserve">4HAR</t>
   </si>
   <si>
     <t xml:space="preserve">2-96 (100)</t>
   </si>
   <si>
-    <t xml:space="preserve">5wf1</t>
+    <t xml:space="preserve">5WF1</t>
   </si>
   <si>
     <t xml:space="preserve">16-116 (120)</t>
@@ -915,7 +915,7 @@
     <t xml:space="preserve">21-104 (115)</t>
   </si>
   <si>
-    <t xml:space="preserve">2qrw</t>
+    <t xml:space="preserve">2QRW</t>
   </si>
   <si>
     <t xml:space="preserve"> Mycobacterium tuberculosis </t>
@@ -924,13 +924,13 @@
     <t xml:space="preserve">5-123 (127)</t>
   </si>
   <si>
-    <t xml:space="preserve">2gkn</t>
+    <t xml:space="preserve">2GKN</t>
   </si>
   <si>
     <t xml:space="preserve">14-127 (127)</t>
   </si>
   <si>
-    <t xml:space="preserve">4c85</t>
+    <t xml:space="preserve">4C85</t>
   </si>
   <si>
     <t xml:space="preserve"> Danio rerio </t>
@@ -939,13 +939,13 @@
     <t xml:space="preserve">1-138 (138)</t>
   </si>
   <si>
-    <t xml:space="preserve">6u63</t>
+    <t xml:space="preserve">6U63</t>
   </si>
   <si>
     <t xml:space="preserve">18-136 (141)</t>
   </si>
   <si>
-    <t xml:space="preserve">6o4u</t>
+    <t xml:space="preserve">6O4U</t>
   </si>
   <si>
     <t xml:space="preserve">7-113 (120)</t>
@@ -954,13 +954,13 @@
     <t xml:space="preserve">36-141 (146)</t>
   </si>
   <si>
-    <t xml:space="preserve">4xev</t>
+    <t xml:space="preserve">4XEV</t>
   </si>
   <si>
     <t xml:space="preserve">2-136 (147)</t>
   </si>
   <si>
-    <t xml:space="preserve">4mo1</t>
+    <t xml:space="preserve">4MO1</t>
   </si>
   <si>
     <t xml:space="preserve"> Lambdavirus lambda </t>
@@ -972,7 +972,7 @@
     <t xml:space="preserve">1-124 (143)</t>
   </si>
   <si>
-    <t xml:space="preserve">4f07</t>
+    <t xml:space="preserve">4F07</t>
   </si>
   <si>
     <t xml:space="preserve"> Pseudomonas sp. Y2 </t>
@@ -981,7 +981,7 @@
     <t xml:space="preserve">12-137 (151)</t>
   </si>
   <si>
-    <t xml:space="preserve">4zbf</t>
+    <t xml:space="preserve">4ZBF</t>
   </si>
   <si>
     <t xml:space="preserve">6-113 (120)</t>
@@ -996,13 +996,13 @@
     <t xml:space="preserve">5-151 (154)</t>
   </si>
   <si>
-    <t xml:space="preserve">8av9</t>
+    <t xml:space="preserve">8AV9</t>
   </si>
   <si>
     <t xml:space="preserve">46-151 (157)</t>
   </si>
   <si>
-    <t xml:space="preserve">3brp</t>
+    <t xml:space="preserve">3BRP</t>
   </si>
   <si>
     <t xml:space="preserve"> unclassified </t>
@@ -1017,7 +1017,7 @@
     <t xml:space="preserve">27-161 (170)</t>
   </si>
   <si>
-    <t xml:space="preserve">5xqz</t>
+    <t xml:space="preserve">5XQZ</t>
   </si>
   <si>
     <t xml:space="preserve">7-107 (120)</t>
@@ -1026,7 +1026,7 @@
     <t xml:space="preserve">1-178 (178)</t>
   </si>
   <si>
-    <t xml:space="preserve">2np5</t>
+    <t xml:space="preserve">2NP5</t>
   </si>
   <si>
     <t xml:space="preserve"> Rhodococcus jostii RHA1 </t>
@@ -1038,16 +1038,16 @@
     <t xml:space="preserve">63-180 (187)</t>
   </si>
   <si>
-    <t xml:space="preserve">4v54</t>
+    <t xml:space="preserve">4V54</t>
   </si>
   <si>
     <t xml:space="preserve">41-117 (120)</t>
   </si>
   <si>
-    <t xml:space="preserve">7afo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4v65</t>
+    <t xml:space="preserve">7AFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4V65</t>
   </si>
   <si>
     <t xml:space="preserve">41-116 (120)</t>
@@ -1056,7 +1056,7 @@
     <t xml:space="preserve">1-85 (88)</t>
   </si>
   <si>
-    <t xml:space="preserve">1tdp</t>
+    <t xml:space="preserve">1TDP</t>
   </si>
   <si>
     <t xml:space="preserve"> Carnobacterium maltaromaticum </t>
@@ -1068,7 +1068,7 @@
     <t xml:space="preserve">1-111 (111)</t>
   </si>
   <si>
-    <t xml:space="preserve">1bgf</t>
+    <t xml:space="preserve">1BGF</t>
   </si>
   <si>
     <t xml:space="preserve">1-102 (120)</t>
@@ -1077,13 +1077,13 @@
     <t xml:space="preserve">6-116 (124)</t>
   </si>
   <si>
-    <t xml:space="preserve">2gl3</t>
+    <t xml:space="preserve">2GL3</t>
   </si>
   <si>
     <t xml:space="preserve">14-123 (127)</t>
   </si>
   <si>
-    <t xml:space="preserve">1moh</t>
+    <t xml:space="preserve">1MOH</t>
   </si>
   <si>
     <t xml:space="preserve">1-105 (120)</t>
@@ -1092,13 +1092,13 @@
     <t xml:space="preserve">8-132 (142)</t>
   </si>
   <si>
-    <t xml:space="preserve">4zvb</t>
+    <t xml:space="preserve">4ZVB</t>
   </si>
   <si>
     <t xml:space="preserve">22-148 (149)</t>
   </si>
   <si>
-    <t xml:space="preserve">6ybg</t>
+    <t xml:space="preserve">6YBG</t>
   </si>
   <si>
     <t xml:space="preserve">8-113 (120)</t>
@@ -1113,10 +1113,10 @@
     <t xml:space="preserve">38-146 (151)</t>
   </si>
   <si>
-    <t xml:space="preserve">4zva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6ymh</t>
+    <t xml:space="preserve">4ZVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6YMH</t>
   </si>
   <si>
     <t xml:space="preserve">34-153 (153)</t>
@@ -1125,7 +1125,7 @@
     <t xml:space="preserve">35-152 (160)</t>
   </si>
   <si>
-    <t xml:space="preserve">8guo</t>
+    <t xml:space="preserve">8GUO</t>
   </si>
   <si>
     <t xml:space="preserve"> Staphylococcus aureus subsp. aureus NCTC 8325 </t>
@@ -1134,7 +1134,7 @@
     <t xml:space="preserve">11-110 (161)</t>
   </si>
   <si>
-    <t xml:space="preserve">6zsc</t>
+    <t xml:space="preserve">6ZSC</t>
   </si>
   <si>
     <t xml:space="preserve">23-118 (120)</t>
@@ -1143,7 +1143,7 @@
     <t xml:space="preserve">1-122 (164)</t>
   </si>
   <si>
-    <t xml:space="preserve">3j9m</t>
+    <t xml:space="preserve">3J9M</t>
   </si>
   <si>
     <t xml:space="preserve">3-115 (120)</t>
@@ -1152,7 +1152,7 @@
     <t xml:space="preserve">1-121 (164)</t>
   </si>
   <si>
-    <t xml:space="preserve">3gw4</t>
+    <t xml:space="preserve">3GW4</t>
   </si>
   <si>
     <t xml:space="preserve"> Deinococcus radiodurans R1 = ATCC 13939 = DSM 20539 </t>
@@ -1164,7 +1164,7 @@
     <t xml:space="preserve">32-182 (192)</t>
   </si>
   <si>
-    <t xml:space="preserve">2i51</t>
+    <t xml:space="preserve">2I51</t>
   </si>
   <si>
     <t xml:space="preserve"> Nostoc punctiforme PCC 73102 </t>
@@ -1173,7 +1173,7 @@
     <t xml:space="preserve">25-176 (191)</t>
   </si>
   <si>
-    <t xml:space="preserve">2n01</t>
+    <t xml:space="preserve">2N01</t>
   </si>
   <si>
     <t xml:space="preserve"> Xanthomonas citri pv. citri str. 306 </t>
@@ -1182,7 +1182,7 @@
     <t xml:space="preserve">16-104 (106)</t>
   </si>
   <si>
-    <t xml:space="preserve">1unn</t>
+    <t xml:space="preserve">1UNN</t>
   </si>
   <si>
     <t xml:space="preserve">4-115 (120)</t>
@@ -1191,7 +1191,7 @@
     <t xml:space="preserve">1-97 (111)</t>
   </si>
   <si>
-    <t xml:space="preserve">3aq8</t>
+    <t xml:space="preserve">3AQ8</t>
   </si>
   <si>
     <t xml:space="preserve"> Tetrahymena pyriformis </t>
@@ -1203,7 +1203,7 @@
     <t xml:space="preserve">2-115 (117)</t>
   </si>
   <si>
-    <t xml:space="preserve">7oom</t>
+    <t xml:space="preserve">7OOM</t>
   </si>
   <si>
     <t xml:space="preserve"> Trichonephila clavipes </t>
@@ -1215,7 +1215,7 @@
     <t xml:space="preserve">15-122 (125)</t>
   </si>
   <si>
-    <t xml:space="preserve">3oj6</t>
+    <t xml:space="preserve">3OJ6</t>
   </si>
   <si>
     <t xml:space="preserve"> Coccidioides immitis </t>
@@ -1224,7 +1224,7 @@
     <t xml:space="preserve">4-118 (128)</t>
   </si>
   <si>
-    <t xml:space="preserve">1b0b</t>
+    <t xml:space="preserve">1B0B</t>
   </si>
   <si>
     <t xml:space="preserve">24-120 (120)</t>
@@ -1233,7 +1233,7 @@
     <t xml:space="preserve">10-136 (142)</t>
   </si>
   <si>
-    <t xml:space="preserve">7ezx</t>
+    <t xml:space="preserve">7EZX</t>
   </si>
   <si>
     <t xml:space="preserve"> Porphyridium purpureum </t>
@@ -1242,7 +1242,7 @@
     <t xml:space="preserve">7-108 (145)</t>
   </si>
   <si>
-    <t xml:space="preserve">5jv4</t>
+    <t xml:space="preserve">5JV4</t>
   </si>
   <si>
     <t xml:space="preserve"> Mycolicibacterium smegmatis </t>
@@ -1254,7 +1254,7 @@
     <t xml:space="preserve">10-92 (138)</t>
   </si>
   <si>
-    <t xml:space="preserve">3wpx</t>
+    <t xml:space="preserve">3WPX</t>
   </si>
   <si>
     <t xml:space="preserve"> Vibrio alginolyticus </t>
@@ -1266,13 +1266,13 @@
     <t xml:space="preserve">9-141 (148)</t>
   </si>
   <si>
-    <t xml:space="preserve">1wv4</t>
+    <t xml:space="preserve">1WV4</t>
   </si>
   <si>
     <t xml:space="preserve">34-153 (154)</t>
   </si>
   <si>
-    <t xml:space="preserve">6i2z</t>
+    <t xml:space="preserve">6I2Z</t>
   </si>
   <si>
     <t xml:space="preserve"> Bordetella pertussis Tohama I </t>
@@ -1281,7 +1281,7 @@
     <t xml:space="preserve">24-144 (151)</t>
   </si>
   <si>
-    <t xml:space="preserve">8csr</t>
+    <t xml:space="preserve">8CSR</t>
   </si>
   <si>
     <t xml:space="preserve">23-119 (120)</t>
@@ -1296,7 +1296,7 @@
     <t xml:space="preserve">40-160 (162)</t>
   </si>
   <si>
-    <t xml:space="preserve">4jiz</t>
+    <t xml:space="preserve">4JIZ</t>
   </si>
   <si>
     <t xml:space="preserve">34-118 (120)</t>
@@ -1305,7 +1305,7 @@
     <t xml:space="preserve">27-164 (172)</t>
   </si>
   <si>
-    <t xml:space="preserve">7vw1</t>
+    <t xml:space="preserve">7VW1</t>
   </si>
   <si>
     <t xml:space="preserve">23-113 (120)</t>
@@ -1314,7 +1314,7 @@
     <t xml:space="preserve">9-85 (92)</t>
   </si>
   <si>
-    <t xml:space="preserve">8g4p</t>
+    <t xml:space="preserve">8G4P</t>
   </si>
   <si>
     <t xml:space="preserve"> Arachis hypogaea </t>
@@ -1326,7 +1326,7 @@
     <t xml:space="preserve">18-90 (94)</t>
   </si>
   <si>
-    <t xml:space="preserve">3r2n</t>
+    <t xml:space="preserve">3R2N</t>
   </si>
   <si>
     <t xml:space="preserve"> Mycobacterium leprae Br4923 </t>
@@ -1338,7 +1338,7 @@
     <t xml:space="preserve">6-119 (119)</t>
   </si>
   <si>
-    <t xml:space="preserve">7d2w</t>
+    <t xml:space="preserve">7D2W</t>
   </si>
   <si>
     <t xml:space="preserve">25-119 (120)</t>
@@ -1347,7 +1347,7 @@
     <t xml:space="preserve">4-113 (125)</t>
   </si>
   <si>
-    <t xml:space="preserve">5e7t</t>
+    <t xml:space="preserve">5E7T</t>
   </si>
   <si>
     <t xml:space="preserve"> Lactococcus phage Tuc2009 </t>
@@ -1356,19 +1356,19 @@
     <t xml:space="preserve">17-95 (129)</t>
   </si>
   <si>
-    <t xml:space="preserve">3wix</t>
+    <t xml:space="preserve">3WIX</t>
   </si>
   <si>
     <t xml:space="preserve">8-140 (144)</t>
   </si>
   <si>
-    <t xml:space="preserve">5fdr</t>
+    <t xml:space="preserve">5FDR</t>
   </si>
   <si>
     <t xml:space="preserve">9-144 (149)</t>
   </si>
   <si>
-    <t xml:space="preserve">2hq9</t>
+    <t xml:space="preserve">2HQ9</t>
   </si>
   <si>
     <t xml:space="preserve"> Mesorhizobium loti </t>
@@ -1377,7 +1377,7 @@
     <t xml:space="preserve">19-135 (138)</t>
   </si>
   <si>
-    <t xml:space="preserve">2hq7</t>
+    <t xml:space="preserve">2HQ7</t>
   </si>
   <si>
     <t xml:space="preserve"> Clostridium acetobutylicum </t>
@@ -1386,7 +1386,7 @@
     <t xml:space="preserve">16-128 (142)</t>
   </si>
   <si>
-    <t xml:space="preserve">8eup</t>
+    <t xml:space="preserve">8EUP</t>
   </si>
   <si>
     <t xml:space="preserve"> Schizosaccharomyces pombe </t>
@@ -1398,7 +1398,7 @@
     <t xml:space="preserve">1-102 (151)</t>
   </si>
   <si>
-    <t xml:space="preserve">3pmd</t>
+    <t xml:space="preserve">3PMD</t>
   </si>
   <si>
     <t xml:space="preserve"> Bacillus anthracis </t>
@@ -1410,7 +1410,7 @@
     <t xml:space="preserve">5-131 (153)</t>
   </si>
   <si>
-    <t xml:space="preserve">7qsf</t>
+    <t xml:space="preserve">7QSF</t>
   </si>
   <si>
     <t xml:space="preserve">24-112 (120)</t>
@@ -1419,7 +1419,7 @@
     <t xml:space="preserve">21-111 (152)</t>
   </si>
   <si>
-    <t xml:space="preserve">6s18</t>
+    <t xml:space="preserve">6S18</t>
   </si>
   <si>
     <t xml:space="preserve"> Pseudomonas putida KT2440 </t>
@@ -1431,13 +1431,13 @@
     <t xml:space="preserve">9-101 (143)</t>
   </si>
   <si>
-    <t xml:space="preserve">7vw2</t>
+    <t xml:space="preserve">7VW2</t>
   </si>
   <si>
     <t xml:space="preserve">2-78 (85)</t>
   </si>
   <si>
-    <t xml:space="preserve">5arn</t>
+    <t xml:space="preserve">5ARN</t>
   </si>
   <si>
     <t xml:space="preserve"> Methylosinus trichosporium OB3b </t>
@@ -1449,7 +1449,7 @@
     <t xml:space="preserve">1-108 (116)</t>
   </si>
   <si>
-    <t xml:space="preserve">1yo7</t>
+    <t xml:space="preserve">1YO7</t>
   </si>
   <si>
     <t xml:space="preserve">6-120 (120)</t>
@@ -1461,19 +1461,19 @@
     <t xml:space="preserve">22-117 (120)</t>
   </si>
   <si>
-    <t xml:space="preserve">3dlq</t>
+    <t xml:space="preserve">3DLQ</t>
   </si>
   <si>
     <t xml:space="preserve">11-131 (131)</t>
   </si>
   <si>
-    <t xml:space="preserve">3esk</t>
+    <t xml:space="preserve">3ESK</t>
   </si>
   <si>
     <t xml:space="preserve">15-117 (128)</t>
   </si>
   <si>
-    <t xml:space="preserve">4yo5</t>
+    <t xml:space="preserve">4YO5</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia coli 042 </t>
@@ -1485,13 +1485,13 @@
     <t xml:space="preserve">49-128 (131)</t>
   </si>
   <si>
-    <t xml:space="preserve">1r5t</t>
+    <t xml:space="preserve">1R5T</t>
   </si>
   <si>
     <t xml:space="preserve">11-133 (134)</t>
   </si>
   <si>
-    <t xml:space="preserve">3cp3</t>
+    <t xml:space="preserve">3CP3</t>
   </si>
   <si>
     <t xml:space="preserve"> Corynebacterium diphtheriae NCTC 13129 </t>
@@ -1500,7 +1500,7 @@
     <t xml:space="preserve">18-124 (127)</t>
   </si>
   <si>
-    <t xml:space="preserve">2hhz</t>
+    <t xml:space="preserve">2HHZ</t>
   </si>
   <si>
     <t xml:space="preserve"> Streptococcus suis 89/1591 </t>
@@ -1512,13 +1512,13 @@
     <t xml:space="preserve">13-134 (139)</t>
   </si>
   <si>
-    <t xml:space="preserve">5lnf</t>
+    <t xml:space="preserve">5LNF</t>
   </si>
   <si>
     <t xml:space="preserve">34-121 (139)</t>
   </si>
   <si>
-    <t xml:space="preserve">3t48</t>
+    <t xml:space="preserve">3T48</t>
   </si>
   <si>
     <t xml:space="preserve"> Staphylococcus aureus subsp. aureus Mu50 </t>
@@ -1527,13 +1527,13 @@
     <t xml:space="preserve">9-66 (70)</t>
   </si>
   <si>
-    <t xml:space="preserve">6stj</t>
+    <t xml:space="preserve">6STJ</t>
   </si>
   <si>
     <t xml:space="preserve">17-99 (103)</t>
   </si>
   <si>
-    <t xml:space="preserve">4ue0</t>
+    <t xml:space="preserve">4UE0</t>
   </si>
   <si>
     <t xml:space="preserve"> Bovine adenovirus 4 </t>
@@ -1542,7 +1542,7 @@
     <t xml:space="preserve">15-114 (115)</t>
   </si>
   <si>
-    <t xml:space="preserve">4wif</t>
+    <t xml:space="preserve">4WIF</t>
   </si>
   <si>
     <t xml:space="preserve">16-109 (120)</t>
@@ -1551,7 +1551,7 @@
     <t xml:space="preserve">1-114 (122)</t>
   </si>
   <si>
-    <t xml:space="preserve">1ux0</t>
+    <t xml:space="preserve">1UX0</t>
   </si>
   <si>
     <t xml:space="preserve"> Bacillus subtilis </t>
@@ -1560,19 +1560,19 @@
     <t xml:space="preserve">1-128 (130)</t>
   </si>
   <si>
-    <t xml:space="preserve">1jtk</t>
+    <t xml:space="preserve">1JTK</t>
   </si>
   <si>
     <t xml:space="preserve">1-128 (131)</t>
   </si>
   <si>
-    <t xml:space="preserve">2fr6</t>
+    <t xml:space="preserve">2FR6</t>
   </si>
   <si>
     <t xml:space="preserve">8-128 (137)</t>
   </si>
   <si>
-    <t xml:space="preserve">7vy1</t>
+    <t xml:space="preserve">7VY1</t>
   </si>
   <si>
     <t xml:space="preserve"> Sus scrofa </t>
@@ -1581,13 +1581,13 @@
     <t xml:space="preserve">2-69 (129)</t>
   </si>
   <si>
-    <t xml:space="preserve">1ux1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7v2f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2fhq</t>
+    <t xml:space="preserve">1UX1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7V2F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2FHQ</t>
   </si>
   <si>
     <t xml:space="preserve"> Bacteroides thetaiotaomicron VPI-5482 </t>
@@ -1596,7 +1596,7 @@
     <t xml:space="preserve">14-134 (134)</t>
   </si>
   <si>
-    <t xml:space="preserve">1uwz</t>
+    <t xml:space="preserve">1UWZ</t>
   </si>
   <si>
     <t xml:space="preserve">3-108 (120)</t>
@@ -1605,7 +1605,7 @@
     <t xml:space="preserve">1-118 (130)</t>
   </si>
   <si>
-    <t xml:space="preserve">6qc4</t>
+    <t xml:space="preserve">6QC4</t>
   </si>
   <si>
     <t xml:space="preserve"> Ovis aries </t>
@@ -1614,7 +1614,7 @@
     <t xml:space="preserve">23-135 (140)</t>
   </si>
   <si>
-    <t xml:space="preserve">5mmm</t>
+    <t xml:space="preserve">5MMM</t>
   </si>
   <si>
     <t xml:space="preserve"> Spinacia oleracea </t>
@@ -1626,7 +1626,7 @@
     <t xml:space="preserve">1-69 (75)</t>
   </si>
   <si>
-    <t xml:space="preserve">6rur</t>
+    <t xml:space="preserve">6RUR</t>
   </si>
   <si>
     <t xml:space="preserve"> Staphylococcus aureus </t>
@@ -1638,7 +1638,7 @@
     <t xml:space="preserve">26-80 (84)</t>
   </si>
   <si>
-    <t xml:space="preserve">7dms</t>
+    <t xml:space="preserve">7DMS</t>
   </si>
   <si>
     <t xml:space="preserve"> Yersinia pseudotuberculosis IP 32953 </t>
@@ -1647,7 +1647,7 @@
     <t xml:space="preserve">9-88 (94)</t>
   </si>
   <si>
-    <t xml:space="preserve">5n5e</t>
+    <t xml:space="preserve">5N5E</t>
   </si>
   <si>
     <t xml:space="preserve"> Pyrococcus furiosus COM1 </t>
@@ -1659,13 +1659,13 @@
     <t xml:space="preserve">15-98 (98)</t>
   </si>
   <si>
-    <t xml:space="preserve">4j2c</t>
+    <t xml:space="preserve">4J2C</t>
   </si>
   <si>
     <t xml:space="preserve">6-104 (106)</t>
   </si>
   <si>
-    <t xml:space="preserve">1nwm</t>
+    <t xml:space="preserve">1NWM</t>
   </si>
   <si>
     <t xml:space="preserve">25-112 (120)</t>
@@ -1674,7 +1674,7 @@
     <t xml:space="preserve">17-100 (105)</t>
   </si>
   <si>
-    <t xml:space="preserve">3sjr</t>
+    <t xml:space="preserve">3SJR</t>
   </si>
   <si>
     <t xml:space="preserve"> Chromobacterium violaceum </t>
@@ -1686,7 +1686,7 @@
     <t xml:space="preserve">9-115 (117)</t>
   </si>
   <si>
-    <t xml:space="preserve">5aqj</t>
+    <t xml:space="preserve">5AQJ</t>
   </si>
   <si>
     <t xml:space="preserve">20-93 (120)</t>
@@ -1695,7 +1695,7 @@
     <t xml:space="preserve">14-112 (112)</t>
   </si>
   <si>
-    <t xml:space="preserve">5aqt</t>
+    <t xml:space="preserve">5AQT</t>
   </si>
   <si>
     <t xml:space="preserve">31-120 (120)</t>
@@ -1704,7 +1704,7 @@
     <t xml:space="preserve">12-114 (115)</t>
   </si>
   <si>
-    <t xml:space="preserve">5l89</t>
+    <t xml:space="preserve">5L89</t>
   </si>
   <si>
     <t xml:space="preserve"> Rhodospirillum rubrum </t>
@@ -1716,7 +1716,7 @@
     <t xml:space="preserve">1-74 (83)</t>
   </si>
   <si>
-    <t xml:space="preserve">6suw</t>
+    <t xml:space="preserve">6SUW</t>
   </si>
   <si>
     <t xml:space="preserve"> Rhodospirillum rubrum ATCC 11170 </t>
@@ -1725,7 +1725,7 @@
     <t xml:space="preserve">11-89 (89)</t>
   </si>
   <si>
-    <t xml:space="preserve">2q9l</t>
+    <t xml:space="preserve">2Q9L</t>
   </si>
   <si>
     <t xml:space="preserve"> Vibrio sp. DAT722 </t>
@@ -1740,10 +1740,10 @@
     <t xml:space="preserve">11-89 (91)</t>
   </si>
   <si>
-    <t xml:space="preserve">6sv1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5l8b</t>
+    <t xml:space="preserve">6SV1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5L8B</t>
   </si>
   <si>
     <t xml:space="preserve">33-112 (120)</t>
@@ -1752,7 +1752,7 @@
     <t xml:space="preserve">12-89 (90)</t>
   </si>
   <si>
-    <t xml:space="preserve">6v3e</t>
+    <t xml:space="preserve">6V3E</t>
   </si>
   <si>
     <t xml:space="preserve"> Acinetobacter baumannii AB0057 </t>
@@ -1761,10 +1761,10 @@
     <t xml:space="preserve">12-89 (91)</t>
   </si>
   <si>
-    <t xml:space="preserve">5l8g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6ehp</t>
+    <t xml:space="preserve">5L8G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6EHP</t>
   </si>
   <si>
     <t xml:space="preserve">2-111 (120)</t>
@@ -1773,19 +1773,19 @@
     <t xml:space="preserve">26-89 (91)</t>
   </si>
   <si>
-    <t xml:space="preserve">5l8f</t>
+    <t xml:space="preserve">5L8F</t>
   </si>
   <si>
     <t xml:space="preserve">11-88 (91)</t>
   </si>
   <si>
-    <t xml:space="preserve">5uyq</t>
+    <t xml:space="preserve">5UYQ</t>
   </si>
   <si>
     <t xml:space="preserve">19-85 (85)</t>
   </si>
   <si>
-    <t xml:space="preserve">7dgw</t>
+    <t xml:space="preserve">7DGW</t>
   </si>
   <si>
     <t xml:space="preserve"> Escherichia coli 'BL21-Gold(DE3)pLysS AG' </t>
@@ -1812,7 +1812,7 @@
     <t xml:space="preserve">10-82 (88)</t>
   </si>
   <si>
-    <t xml:space="preserve">4adz</t>
+    <t xml:space="preserve">4ADZ</t>
   </si>
   <si>
     <t xml:space="preserve"> Streptomyces lividans </t>
@@ -1824,7 +1824,7 @@
     <t xml:space="preserve">1-90 (90)</t>
   </si>
   <si>
-    <t xml:space="preserve">6zkg</t>
+    <t xml:space="preserve">6ZKG</t>
   </si>
   <si>
     <t xml:space="preserve">20-94 (120)</t>
@@ -1833,13 +1833,13 @@
     <t xml:space="preserve">9-78 (98)</t>
   </si>
   <si>
-    <t xml:space="preserve">5aqq</t>
+    <t xml:space="preserve">5AQQ</t>
   </si>
   <si>
     <t xml:space="preserve">13-108 (108)</t>
   </si>
   <si>
-    <t xml:space="preserve">5z8q</t>
+    <t xml:space="preserve">5Z8Q</t>
   </si>
   <si>
     <t xml:space="preserve"> Saccharomyces cerevisiae S288C </t>
@@ -1848,7 +1848,7 @@
     <t xml:space="preserve">17-81 (101)</t>
   </si>
   <si>
-    <t xml:space="preserve">5j0l</t>
+    <t xml:space="preserve">5J0L</t>
   </si>
   <si>
     <t xml:space="preserve">31-118 (120)</t>
@@ -1857,7 +1857,7 @@
     <t xml:space="preserve">3-99 (111)</t>
   </si>
   <si>
-    <t xml:space="preserve">1hx1</t>
+    <t xml:space="preserve">1HX1</t>
   </si>
   <si>
     <t xml:space="preserve">27-112 (120)</t>
@@ -1866,13 +1866,13 @@
     <t xml:space="preserve">7-104 (112)</t>
   </si>
   <si>
-    <t xml:space="preserve">5hy3</t>
+    <t xml:space="preserve">5HY3</t>
   </si>
   <si>
     <t xml:space="preserve">2-48 (57)</t>
   </si>
   <si>
-    <t xml:space="preserve">8szz</t>
+    <t xml:space="preserve">8SZZ</t>
   </si>
   <si>
     <t xml:space="preserve">60-112 (120)</t>
@@ -1881,7 +1881,7 @@
     <t xml:space="preserve">11-60 (70)</t>
   </si>
   <si>
-    <t xml:space="preserve">3lof</t>
+    <t xml:space="preserve">3LOF</t>
   </si>
   <si>
     <t xml:space="preserve">4-112 (120)</t>
@@ -1896,13 +1896,13 @@
     <t xml:space="preserve">11-83 (84)</t>
   </si>
   <si>
-    <t xml:space="preserve">2qj9</t>
+    <t xml:space="preserve">2QJ9</t>
   </si>
   <si>
     <t xml:space="preserve">3-83 (86)</t>
   </si>
   <si>
-    <t xml:space="preserve">3nkz</t>
+    <t xml:space="preserve">3NKZ</t>
   </si>
   <si>
     <t xml:space="preserve"> Yersinia enterocolitica subsp. enterocolitica 8081 </t>
@@ -1914,7 +1914,7 @@
     <t xml:space="preserve">10-84 (95)</t>
   </si>
   <si>
-    <t xml:space="preserve">4fi5</t>
+    <t xml:space="preserve">4FI5</t>
   </si>
   <si>
     <t xml:space="preserve"> Hantaan virus 76-118 </t>
@@ -1923,7 +1923,7 @@
     <t xml:space="preserve">11-60 (71)</t>
   </si>
   <si>
-    <t xml:space="preserve">6dlm</t>
+    <t xml:space="preserve">6DLM</t>
   </si>
   <si>
     <t xml:space="preserve">61-111 (120)</t>
@@ -1932,7 +1932,7 @@
     <t xml:space="preserve">18-59 (74)</t>
   </si>
   <si>
-    <t xml:space="preserve">7mkk</t>
+    <t xml:space="preserve">7MKK</t>
   </si>
   <si>
     <t xml:space="preserve"> Drosophila melanogaster </t>
@@ -1941,7 +1941,7 @@
     <t xml:space="preserve">5-70 (71)</t>
   </si>
   <si>
-    <t xml:space="preserve">5j73</t>
+    <t xml:space="preserve">5J73</t>
   </si>
   <si>
     <t xml:space="preserve">1-82 (120)</t>
@@ -1950,7 +1950,7 @@
     <t xml:space="preserve">5-73 (73)</t>
   </si>
   <si>
-    <t xml:space="preserve">1ijc</t>
+    <t xml:space="preserve">1IJC</t>
   </si>
   <si>
     <t xml:space="preserve"> Bungarus candidus </t>
@@ -1962,7 +1962,7 @@
     <t xml:space="preserve">1-63 (63)</t>
   </si>
   <si>
-    <t xml:space="preserve">6wa9</t>
+    <t xml:space="preserve">6WA9</t>
   </si>
   <si>
     <t xml:space="preserve"> Chlamydia pneumoniae </t>
@@ -1971,7 +1971,7 @@
     <t xml:space="preserve">23-68 (83)</t>
   </si>
   <si>
-    <t xml:space="preserve">6inr</t>
+    <t xml:space="preserve">6INR</t>
   </si>
   <si>
     <t xml:space="preserve"> 'Echinacea purpurea' witches'-broom phytoplasma </t>
@@ -1983,7 +1983,7 @@
     <t xml:space="preserve">16-54 (69)</t>
   </si>
   <si>
-    <t xml:space="preserve">8i9r</t>
+    <t xml:space="preserve">8I9R</t>
   </si>
   <si>
     <t xml:space="preserve"> Thermochaetoides thermophila DSM 1495 </t>
@@ -1995,7 +1995,7 @@
     <t xml:space="preserve">20-71 (71)</t>
   </si>
   <si>
-    <t xml:space="preserve">7p47</t>
+    <t xml:space="preserve">7P47</t>
   </si>
   <si>
     <t xml:space="preserve">18-56 (69)</t>
@@ -2084,7 +2084,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -2101,6 +2101,13 @@
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -2129,7 +2136,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2142,7 +2149,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2175,6 +2182,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8042,25 +8069,25 @@
       <c r="H234" s="11"/>
     </row>
     <row r="235" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A235" s="6" t="s">
+      <c r="A235" s="12" t="s">
         <v>651</v>
       </c>
-      <c r="B235" s="7" t="s">
+      <c r="B235" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="C235" s="8" t="n">
+      <c r="C235" s="14" t="n">
         <v>0.04</v>
       </c>
-      <c r="D235" s="8" t="n">
+      <c r="D235" s="14" t="n">
         <v>0.303</v>
       </c>
-      <c r="E235" s="9" t="n">
+      <c r="E235" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="F235" s="10" t="s">
+      <c r="F235" s="16" t="s">
         <v>645</v>
       </c>
-      <c r="G235" s="10" t="s">
+      <c r="G235" s="16" t="s">
         <v>652</v>
       </c>
       <c r="H235" s="11"/>

</xml_diff>